<commit_message>
Label downtilt/uptilt recommendations with coverage effect
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018bjY7UMi7f9uTvsfcag3Vv
</commit_message>
<xml_diff>
--- a/Terrain_Clutter_RF_Recommendation_Filled.xlsx
+++ b/Terrain_Clutter_RF_Recommendation_Filled.xlsx
@@ -629,17 +629,17 @@
       </c>
       <c r="D2" s="7" t="inlineStr">
         <is>
-          <t>+2° Downtilt</t>
+          <t>+2° Downtilt (Reduce Coverage)</t>
         </is>
       </c>
       <c r="E2" s="7" t="inlineStr">
         <is>
-          <t>+1° Downtilt</t>
+          <t>+1° Downtilt (Reduce Coverage)</t>
         </is>
       </c>
       <c r="F2" s="7" t="inlineStr">
         <is>
-          <t>+1° Downtilt (facing cells only)</t>
+          <t>+1° Downtilt (Reduce Coverage – facing cells only)</t>
         </is>
       </c>
       <c r="G2" s="8" t="inlineStr">
@@ -666,7 +666,7 @@
       </c>
       <c r="D3" s="7" t="inlineStr">
         <is>
-          <t>-1° Uptilt</t>
+          <t>-1° Uptilt (Increase Coverage)</t>
         </is>
       </c>
       <c r="E3" s="7" t="inlineStr">
@@ -703,12 +703,12 @@
       </c>
       <c r="D4" s="10" t="inlineStr">
         <is>
-          <t>+2° Downtilt</t>
+          <t>+2° Downtilt (Reduce Coverage)</t>
         </is>
       </c>
       <c r="E4" s="10" t="inlineStr">
         <is>
-          <t>+1° Downtilt</t>
+          <t>+1° Downtilt (Reduce Coverage)</t>
         </is>
       </c>
       <c r="F4" s="10" t="inlineStr">
@@ -740,7 +740,7 @@
       </c>
       <c r="D5" s="10" t="inlineStr">
         <is>
-          <t>-1° Uptilt</t>
+          <t>-1° Uptilt (Increase Coverage)</t>
         </is>
       </c>
       <c r="E5" s="10" t="inlineStr">
@@ -750,7 +750,7 @@
       </c>
       <c r="F5" s="10" t="inlineStr">
         <is>
-          <t>-1° Uptilt (cell facing gap only)</t>
+          <t>-1° Uptilt (Increase Coverage – cell facing gap only)</t>
         </is>
       </c>
       <c r="G5" s="11" t="inlineStr">
@@ -777,7 +777,7 @@
       </c>
       <c r="D6" s="7" t="inlineStr">
         <is>
-          <t>+2° Downtilt</t>
+          <t>+2° Downtilt (Reduce Coverage)</t>
         </is>
       </c>
       <c r="E6" s="7" t="inlineStr">
@@ -814,7 +814,7 @@
       </c>
       <c r="D7" s="7" t="inlineStr">
         <is>
-          <t>-2° Uptilt</t>
+          <t>-2° Uptilt (Increase Coverage)</t>
         </is>
       </c>
       <c r="E7" s="7" t="inlineStr">
@@ -824,7 +824,7 @@
       </c>
       <c r="F7" s="7" t="inlineStr">
         <is>
-          <t>-1° Uptilt (facing cells only)</t>
+          <t>-1° Uptilt (Increase Coverage – facing cells only)</t>
         </is>
       </c>
       <c r="G7" s="8" t="inlineStr">
@@ -851,7 +851,7 @@
       </c>
       <c r="D8" s="10" t="inlineStr">
         <is>
-          <t>+1° Downtilt</t>
+          <t>+1° Downtilt (Reduce Coverage)</t>
         </is>
       </c>
       <c r="E8" s="10" t="inlineStr">
@@ -888,12 +888,12 @@
       </c>
       <c r="D9" s="10" t="inlineStr">
         <is>
-          <t>-2° Uptilt</t>
+          <t>-2° Uptilt (Increase Coverage)</t>
         </is>
       </c>
       <c r="E9" s="10" t="inlineStr">
         <is>
-          <t>-1° Uptilt</t>
+          <t>-1° Uptilt (Increase Coverage)</t>
         </is>
       </c>
       <c r="F9" s="10" t="inlineStr">
@@ -925,7 +925,7 @@
       </c>
       <c r="D10" s="7" t="inlineStr">
         <is>
-          <t>+1° Downtilt</t>
+          <t>+1° Downtilt (Reduce Coverage)</t>
         </is>
       </c>
       <c r="E10" s="7" t="inlineStr">
@@ -962,12 +962,12 @@
       </c>
       <c r="D11" s="7" t="inlineStr">
         <is>
-          <t>-2° Uptilt</t>
+          <t>-2° Uptilt (Increase Coverage)</t>
         </is>
       </c>
       <c r="E11" s="7" t="inlineStr">
         <is>
-          <t>-1° Uptilt</t>
+          <t>-1° Uptilt (Increase Coverage)</t>
         </is>
       </c>
       <c r="F11" s="7" t="inlineStr">
@@ -999,17 +999,17 @@
       </c>
       <c r="D12" s="10" t="inlineStr">
         <is>
-          <t>+3° Downtilt</t>
+          <t>+3° Downtilt (Reduce Coverage)</t>
         </is>
       </c>
       <c r="E12" s="10" t="inlineStr">
         <is>
-          <t>+1° Downtilt</t>
+          <t>+1° Downtilt (Reduce Coverage)</t>
         </is>
       </c>
       <c r="F12" s="10" t="inlineStr">
         <is>
-          <t>+1° Downtilt (cells facing open area)</t>
+          <t>+1° Downtilt (Reduce Coverage – cells facing open area)</t>
         </is>
       </c>
       <c r="G12" s="11" t="inlineStr">
@@ -1036,7 +1036,7 @@
       </c>
       <c r="D13" s="10" t="inlineStr">
         <is>
-          <t>-2° Uptilt</t>
+          <t>-2° Uptilt (Increase Coverage)</t>
         </is>
       </c>
       <c r="E13" s="10" t="inlineStr">
@@ -1073,17 +1073,17 @@
       </c>
       <c r="D14" s="10" t="inlineStr">
         <is>
-          <t>+2° Downtilt</t>
+          <t>+2° Downtilt (Reduce Coverage)</t>
         </is>
       </c>
       <c r="E14" s="10" t="inlineStr">
         <is>
-          <t>+1° Downtilt</t>
+          <t>+1° Downtilt (Reduce Coverage)</t>
         </is>
       </c>
       <c r="F14" s="10" t="inlineStr">
         <is>
-          <t>+1° Downtilt (facing cells only)</t>
+          <t>+1° Downtilt (Reduce Coverage – facing cells only)</t>
         </is>
       </c>
       <c r="G14" s="11" t="inlineStr">
@@ -1110,7 +1110,7 @@
       </c>
       <c r="D15" s="10" t="inlineStr">
         <is>
-          <t>-1° Uptilt</t>
+          <t>-1° Uptilt (Increase Coverage)</t>
         </is>
       </c>
       <c r="E15" s="10" t="inlineStr">
@@ -1147,12 +1147,12 @@
       </c>
       <c r="D16" s="7" t="inlineStr">
         <is>
-          <t>+2° Downtilt</t>
+          <t>+2° Downtilt (Reduce Coverage)</t>
         </is>
       </c>
       <c r="E16" s="7" t="inlineStr">
         <is>
-          <t>+1° Downtilt</t>
+          <t>+1° Downtilt (Reduce Coverage)</t>
         </is>
       </c>
       <c r="F16" s="7" t="inlineStr">
@@ -1184,7 +1184,7 @@
       </c>
       <c r="D17" s="7" t="inlineStr">
         <is>
-          <t>-1° Uptilt</t>
+          <t>-1° Uptilt (Increase Coverage)</t>
         </is>
       </c>
       <c r="E17" s="7" t="inlineStr">
@@ -1194,7 +1194,7 @@
       </c>
       <c r="F17" s="7" t="inlineStr">
         <is>
-          <t>-1° Uptilt (cell facing gap only)</t>
+          <t>-1° Uptilt (Increase Coverage – cell facing gap only)</t>
         </is>
       </c>
       <c r="G17" s="8" t="inlineStr">
@@ -1221,7 +1221,7 @@
       </c>
       <c r="D18" s="10" t="inlineStr">
         <is>
-          <t>+2° Downtilt</t>
+          <t>+2° Downtilt (Reduce Coverage)</t>
         </is>
       </c>
       <c r="E18" s="10" t="inlineStr">
@@ -1258,7 +1258,7 @@
       </c>
       <c r="D19" s="10" t="inlineStr">
         <is>
-          <t>-2° Uptilt</t>
+          <t>-2° Uptilt (Increase Coverage)</t>
         </is>
       </c>
       <c r="E19" s="10" t="inlineStr">
@@ -1268,7 +1268,7 @@
       </c>
       <c r="F19" s="10" t="inlineStr">
         <is>
-          <t>-1° Uptilt (facing cells only)</t>
+          <t>-1° Uptilt (Increase Coverage – facing cells only)</t>
         </is>
       </c>
       <c r="G19" s="11" t="inlineStr">
@@ -1295,7 +1295,7 @@
       </c>
       <c r="D20" s="7" t="inlineStr">
         <is>
-          <t>+1° Downtilt</t>
+          <t>+1° Downtilt (Reduce Coverage)</t>
         </is>
       </c>
       <c r="E20" s="7" t="inlineStr">
@@ -1332,12 +1332,12 @@
       </c>
       <c r="D21" s="7" t="inlineStr">
         <is>
-          <t>-2° Uptilt</t>
+          <t>-2° Uptilt (Increase Coverage)</t>
         </is>
       </c>
       <c r="E21" s="7" t="inlineStr">
         <is>
-          <t>-1° Uptilt</t>
+          <t>-1° Uptilt (Increase Coverage)</t>
         </is>
       </c>
       <c r="F21" s="7" t="inlineStr">
@@ -1369,7 +1369,7 @@
       </c>
       <c r="D22" s="10" t="inlineStr">
         <is>
-          <t>+1° Downtilt</t>
+          <t>+1° Downtilt (Reduce Coverage)</t>
         </is>
       </c>
       <c r="E22" s="10" t="inlineStr">
@@ -1406,7 +1406,7 @@
       </c>
       <c r="D23" s="10" t="inlineStr">
         <is>
-          <t>-1° Uptilt</t>
+          <t>-1° Uptilt (Increase Coverage)</t>
         </is>
       </c>
       <c r="E23" s="10" t="inlineStr">
@@ -1416,7 +1416,7 @@
       </c>
       <c r="F23" s="10" t="inlineStr">
         <is>
-          <t>-1° Uptilt (facing cells only)</t>
+          <t>-1° Uptilt (Increase Coverage – facing cells only)</t>
         </is>
       </c>
       <c r="G23" s="11" t="inlineStr">
@@ -1443,12 +1443,12 @@
       </c>
       <c r="D24" s="7" t="inlineStr">
         <is>
-          <t>+2° Downtilt</t>
+          <t>+2° Downtilt (Reduce Coverage)</t>
         </is>
       </c>
       <c r="E24" s="7" t="inlineStr">
         <is>
-          <t>+1° Downtilt</t>
+          <t>+1° Downtilt (Reduce Coverage)</t>
         </is>
       </c>
       <c r="F24" s="7" t="inlineStr">
@@ -1480,7 +1480,7 @@
       </c>
       <c r="D25" s="7" t="inlineStr">
         <is>
-          <t>-1° Uptilt</t>
+          <t>-1° Uptilt (Increase Coverage)</t>
         </is>
       </c>
       <c r="E25" s="7" t="inlineStr">
@@ -1517,17 +1517,17 @@
       </c>
       <c r="D26" s="7" t="inlineStr">
         <is>
-          <t>+3° Downtilt</t>
+          <t>+3° Downtilt (Reduce Coverage)</t>
         </is>
       </c>
       <c r="E26" s="7" t="inlineStr">
         <is>
-          <t>+1° Downtilt</t>
+          <t>+1° Downtilt (Reduce Coverage)</t>
         </is>
       </c>
       <c r="F26" s="7" t="inlineStr">
         <is>
-          <t>+1° Downtilt (facing cells only)</t>
+          <t>+1° Downtilt (Reduce Coverage – facing cells only)</t>
         </is>
       </c>
       <c r="G26" s="8" t="inlineStr">
@@ -1554,7 +1554,7 @@
       </c>
       <c r="D27" s="7" t="inlineStr">
         <is>
-          <t>-1° Uptilt (only if gap is in LOS)</t>
+          <t>-1° Uptilt (Increase Coverage – only if gap is in LOS)</t>
         </is>
       </c>
       <c r="E27" s="7" t="inlineStr">
@@ -1564,7 +1564,7 @@
       </c>
       <c r="F27" s="7" t="inlineStr">
         <is>
-          <t>-1° Uptilt (LOS neighbour)</t>
+          <t>-1° Uptilt (Increase Coverage – LOS neighbour)</t>
         </is>
       </c>
       <c r="G27" s="8" t="inlineStr">
@@ -1591,17 +1591,17 @@
       </c>
       <c r="D28" s="10" t="inlineStr">
         <is>
-          <t>+3° Downtilt</t>
+          <t>+3° Downtilt (Reduce Coverage)</t>
         </is>
       </c>
       <c r="E28" s="10" t="inlineStr">
         <is>
-          <t>+1° Downtilt</t>
+          <t>+1° Downtilt (Reduce Coverage)</t>
         </is>
       </c>
       <c r="F28" s="10" t="inlineStr">
         <is>
-          <t>+1° Downtilt (facing cells only)</t>
+          <t>+1° Downtilt (Reduce Coverage – facing cells only)</t>
         </is>
       </c>
       <c r="G28" s="11" t="inlineStr">
@@ -1628,7 +1628,7 @@
       </c>
       <c r="D29" s="10" t="inlineStr">
         <is>
-          <t>-1° Uptilt</t>
+          <t>-1° Uptilt (Increase Coverage)</t>
         </is>
       </c>
       <c r="E29" s="10" t="inlineStr">
@@ -1638,7 +1638,7 @@
       </c>
       <c r="F29" s="10" t="inlineStr">
         <is>
-          <t>-1° Uptilt (LOS neighbour)</t>
+          <t>-1° Uptilt (Increase Coverage – LOS neighbour)</t>
         </is>
       </c>
       <c r="G29" s="11" t="inlineStr">
@@ -1665,12 +1665,12 @@
       </c>
       <c r="D30" s="7" t="inlineStr">
         <is>
-          <t>+2° Downtilt</t>
+          <t>+2° Downtilt (Reduce Coverage)</t>
         </is>
       </c>
       <c r="E30" s="7" t="inlineStr">
         <is>
-          <t>+1° Downtilt</t>
+          <t>+1° Downtilt (Reduce Coverage)</t>
         </is>
       </c>
       <c r="F30" s="7" t="inlineStr">
@@ -1702,7 +1702,7 @@
       </c>
       <c r="D31" s="7" t="inlineStr">
         <is>
-          <t>-1° Uptilt</t>
+          <t>-1° Uptilt (Increase Coverage)</t>
         </is>
       </c>
       <c r="E31" s="7" t="inlineStr">
@@ -1712,7 +1712,7 @@
       </c>
       <c r="F31" s="7" t="inlineStr">
         <is>
-          <t>-1° Uptilt (LOS neighbour)</t>
+          <t>-1° Uptilt (Increase Coverage – LOS neighbour)</t>
         </is>
       </c>
       <c r="G31" s="8" t="inlineStr">
@@ -1739,7 +1739,7 @@
       </c>
       <c r="D32" s="10" t="inlineStr">
         <is>
-          <t>+2° Downtilt</t>
+          <t>+2° Downtilt (Reduce Coverage)</t>
         </is>
       </c>
       <c r="E32" s="10" t="inlineStr">
@@ -1776,7 +1776,7 @@
       </c>
       <c r="D33" s="10" t="inlineStr">
         <is>
-          <t>-1° Uptilt</t>
+          <t>-1° Uptilt (Increase Coverage)</t>
         </is>
       </c>
       <c r="E33" s="10" t="inlineStr">
@@ -1786,7 +1786,7 @@
       </c>
       <c r="F33" s="10" t="inlineStr">
         <is>
-          <t>-1° Uptilt (LOS neighbour)</t>
+          <t>-1° Uptilt (Increase Coverage – LOS neighbour)</t>
         </is>
       </c>
       <c r="G33" s="11" t="inlineStr">
@@ -1813,7 +1813,7 @@
       </c>
       <c r="D34" s="7" t="inlineStr">
         <is>
-          <t>+2° Downtilt</t>
+          <t>+2° Downtilt (Reduce Coverage)</t>
         </is>
       </c>
       <c r="E34" s="7" t="inlineStr">
@@ -1850,7 +1850,7 @@
       </c>
       <c r="D35" s="7" t="inlineStr">
         <is>
-          <t>-1° Uptilt</t>
+          <t>-1° Uptilt (Increase Coverage)</t>
         </is>
       </c>
       <c r="E35" s="7" t="inlineStr">
@@ -1860,7 +1860,7 @@
       </c>
       <c r="F35" s="7" t="inlineStr">
         <is>
-          <t>-1° Uptilt (LOS neighbour)</t>
+          <t>-1° Uptilt (Increase Coverage – LOS neighbour)</t>
         </is>
       </c>
       <c r="G35" s="8" t="inlineStr">
@@ -1887,17 +1887,17 @@
       </c>
       <c r="D36" s="10" t="inlineStr">
         <is>
-          <t>+3° Downtilt</t>
+          <t>+3° Downtilt (Reduce Coverage)</t>
         </is>
       </c>
       <c r="E36" s="10" t="inlineStr">
         <is>
-          <t>+1° Downtilt</t>
+          <t>+1° Downtilt (Reduce Coverage)</t>
         </is>
       </c>
       <c r="F36" s="10" t="inlineStr">
         <is>
-          <t>+1° Downtilt (facing cells only)</t>
+          <t>+1° Downtilt (Reduce Coverage – facing cells only)</t>
         </is>
       </c>
       <c r="G36" s="11" t="inlineStr">
@@ -1924,7 +1924,7 @@
       </c>
       <c r="D37" s="10" t="inlineStr">
         <is>
-          <t>-1° Uptilt</t>
+          <t>-1° Uptilt (Increase Coverage)</t>
         </is>
       </c>
       <c r="E37" s="10" t="inlineStr">
@@ -1961,17 +1961,17 @@
       </c>
       <c r="D38" s="10" t="inlineStr">
         <is>
-          <t>+4° Downtilt</t>
+          <t>+4° Downtilt (Reduce Coverage)</t>
         </is>
       </c>
       <c r="E38" s="10" t="inlineStr">
         <is>
-          <t>+2° Downtilt</t>
+          <t>+2° Downtilt (Reduce Coverage)</t>
         </is>
       </c>
       <c r="F38" s="10" t="inlineStr">
         <is>
-          <t>+2° Downtilt (facing cells)</t>
+          <t>+2° Downtilt (Reduce Coverage – facing cells)</t>
         </is>
       </c>
       <c r="G38" s="11" t="inlineStr">
@@ -2008,7 +2008,7 @@
       </c>
       <c r="F39" s="10" t="inlineStr">
         <is>
-          <t>-1° Uptilt (LOS neighbour across valley)</t>
+          <t>-1° Uptilt (Increase Coverage – LOS neighbour across valley)</t>
         </is>
       </c>
       <c r="G39" s="11" t="inlineStr">
@@ -2035,17 +2035,17 @@
       </c>
       <c r="D40" s="7" t="inlineStr">
         <is>
-          <t>+3° Downtilt</t>
+          <t>+3° Downtilt (Reduce Coverage)</t>
         </is>
       </c>
       <c r="E40" s="7" t="inlineStr">
         <is>
-          <t>+2° Downtilt</t>
+          <t>+2° Downtilt (Reduce Coverage)</t>
         </is>
       </c>
       <c r="F40" s="7" t="inlineStr">
         <is>
-          <t>+1° Downtilt (facing cells)</t>
+          <t>+1° Downtilt (Reduce Coverage – facing cells)</t>
         </is>
       </c>
       <c r="G40" s="8" t="inlineStr">
@@ -2072,7 +2072,7 @@
       </c>
       <c r="D41" s="7" t="inlineStr">
         <is>
-          <t>-1° Uptilt (only if gap is in LOS)</t>
+          <t>-1° Uptilt (Increase Coverage – only if gap is in LOS)</t>
         </is>
       </c>
       <c r="E41" s="7" t="inlineStr">
@@ -2082,7 +2082,7 @@
       </c>
       <c r="F41" s="7" t="inlineStr">
         <is>
-          <t>-1° Uptilt (LOS neighbour)</t>
+          <t>-1° Uptilt (Increase Coverage – LOS neighbour)</t>
         </is>
       </c>
       <c r="G41" s="8" t="inlineStr">
@@ -2109,17 +2109,17 @@
       </c>
       <c r="D42" s="10" t="inlineStr">
         <is>
-          <t>+3° Downtilt</t>
+          <t>+3° Downtilt (Reduce Coverage)</t>
         </is>
       </c>
       <c r="E42" s="10" t="inlineStr">
         <is>
-          <t>+1° Downtilt</t>
+          <t>+1° Downtilt (Reduce Coverage)</t>
         </is>
       </c>
       <c r="F42" s="10" t="inlineStr">
         <is>
-          <t>+1° Downtilt (facing cells)</t>
+          <t>+1° Downtilt (Reduce Coverage – facing cells)</t>
         </is>
       </c>
       <c r="G42" s="11" t="inlineStr">
@@ -2146,7 +2146,7 @@
       </c>
       <c r="D43" s="10" t="inlineStr">
         <is>
-          <t>-1° Uptilt</t>
+          <t>-1° Uptilt (Increase Coverage)</t>
         </is>
       </c>
       <c r="E43" s="10" t="inlineStr">
@@ -2156,7 +2156,7 @@
       </c>
       <c r="F43" s="10" t="inlineStr">
         <is>
-          <t>-1° Uptilt (LOS neighbour)</t>
+          <t>-1° Uptilt (Increase Coverage – LOS neighbour)</t>
         </is>
       </c>
       <c r="G43" s="11" t="inlineStr">
@@ -2183,12 +2183,12 @@
       </c>
       <c r="D44" s="7" t="inlineStr">
         <is>
-          <t>+3° Downtilt</t>
+          <t>+3° Downtilt (Reduce Coverage)</t>
         </is>
       </c>
       <c r="E44" s="7" t="inlineStr">
         <is>
-          <t>+1° Downtilt</t>
+          <t>+1° Downtilt (Reduce Coverage)</t>
         </is>
       </c>
       <c r="F44" s="7" t="inlineStr">
@@ -2220,7 +2220,7 @@
       </c>
       <c r="D45" s="7" t="inlineStr">
         <is>
-          <t>-1° Uptilt</t>
+          <t>-1° Uptilt (Increase Coverage)</t>
         </is>
       </c>
       <c r="E45" s="7" t="inlineStr">
@@ -2257,12 +2257,12 @@
       </c>
       <c r="D46" s="10" t="inlineStr">
         <is>
-          <t>+2° Downtilt</t>
+          <t>+2° Downtilt (Reduce Coverage)</t>
         </is>
       </c>
       <c r="E46" s="10" t="inlineStr">
         <is>
-          <t>+1° Downtilt</t>
+          <t>+1° Downtilt (Reduce Coverage)</t>
         </is>
       </c>
       <c r="F46" s="10" t="inlineStr">
@@ -2294,7 +2294,7 @@
       </c>
       <c r="D47" s="10" t="inlineStr">
         <is>
-          <t>-1° Uptilt</t>
+          <t>-1° Uptilt (Increase Coverage)</t>
         </is>
       </c>
       <c r="E47" s="10" t="inlineStr">
@@ -2304,7 +2304,7 @@
       </c>
       <c r="F47" s="10" t="inlineStr">
         <is>
-          <t>-1° Uptilt (LOS neighbour)</t>
+          <t>-1° Uptilt (Increase Coverage – LOS neighbour)</t>
         </is>
       </c>
       <c r="G47" s="11" t="inlineStr">
@@ -2331,17 +2331,17 @@
       </c>
       <c r="D48" s="7" t="inlineStr">
         <is>
-          <t>+3° Downtilt</t>
+          <t>+3° Downtilt (Reduce Coverage)</t>
         </is>
       </c>
       <c r="E48" s="7" t="inlineStr">
         <is>
-          <t>+1° Downtilt</t>
+          <t>+1° Downtilt (Reduce Coverage)</t>
         </is>
       </c>
       <c r="F48" s="7" t="inlineStr">
         <is>
-          <t>+1° Downtilt (facing cells)</t>
+          <t>+1° Downtilt (Reduce Coverage – facing cells)</t>
         </is>
       </c>
       <c r="G48" s="8" t="inlineStr">
@@ -2368,7 +2368,7 @@
       </c>
       <c r="D49" s="7" t="inlineStr">
         <is>
-          <t>-1° Uptilt</t>
+          <t>-1° Uptilt (Increase Coverage)</t>
         </is>
       </c>
       <c r="E49" s="7" t="inlineStr">
@@ -2405,17 +2405,17 @@
       </c>
       <c r="D50" s="7" t="inlineStr">
         <is>
-          <t>+2° Downtilt</t>
+          <t>+2° Downtilt (Reduce Coverage)</t>
         </is>
       </c>
       <c r="E50" s="7" t="inlineStr">
         <is>
-          <t>+1° Downtilt</t>
+          <t>+1° Downtilt (Reduce Coverage)</t>
         </is>
       </c>
       <c r="F50" s="7" t="inlineStr">
         <is>
-          <t>+1° Downtilt (cells along valley axis)</t>
+          <t>+1° Downtilt (Reduce Coverage – cells along valley axis)</t>
         </is>
       </c>
       <c r="G50" s="8" t="inlineStr">
@@ -2442,7 +2442,7 @@
       </c>
       <c r="D51" s="7" t="inlineStr">
         <is>
-          <t>-1° Uptilt</t>
+          <t>-1° Uptilt (Increase Coverage)</t>
         </is>
       </c>
       <c r="E51" s="7" t="inlineStr">
@@ -2479,17 +2479,17 @@
       </c>
       <c r="D52" s="10" t="inlineStr">
         <is>
-          <t>+2° Downtilt</t>
+          <t>+2° Downtilt (Reduce Coverage)</t>
         </is>
       </c>
       <c r="E52" s="10" t="inlineStr">
         <is>
-          <t>+1° Downtilt</t>
+          <t>+1° Downtilt (Reduce Coverage)</t>
         </is>
       </c>
       <c r="F52" s="10" t="inlineStr">
         <is>
-          <t>+1° Downtilt (cells along valley axis)</t>
+          <t>+1° Downtilt (Reduce Coverage – cells along valley axis)</t>
         </is>
       </c>
       <c r="G52" s="11" t="inlineStr">
@@ -2516,7 +2516,7 @@
       </c>
       <c r="D53" s="10" t="inlineStr">
         <is>
-          <t>-1° Uptilt</t>
+          <t>-1° Uptilt (Increase Coverage)</t>
         </is>
       </c>
       <c r="E53" s="10" t="inlineStr">
@@ -2526,7 +2526,7 @@
       </c>
       <c r="F53" s="10" t="inlineStr">
         <is>
-          <t>-1° Uptilt (cell facing gap only)</t>
+          <t>-1° Uptilt (Increase Coverage – cell facing gap only)</t>
         </is>
       </c>
       <c r="G53" s="11" t="inlineStr">
@@ -2553,12 +2553,12 @@
       </c>
       <c r="D54" s="7" t="inlineStr">
         <is>
-          <t>+2° Downtilt</t>
+          <t>+2° Downtilt (Reduce Coverage)</t>
         </is>
       </c>
       <c r="E54" s="7" t="inlineStr">
         <is>
-          <t>+1° Downtilt</t>
+          <t>+1° Downtilt (Reduce Coverage)</t>
         </is>
       </c>
       <c r="F54" s="7" t="inlineStr">
@@ -2590,7 +2590,7 @@
       </c>
       <c r="D55" s="7" t="inlineStr">
         <is>
-          <t>-2° Uptilt</t>
+          <t>-2° Uptilt (Increase Coverage)</t>
         </is>
       </c>
       <c r="E55" s="7" t="inlineStr">
@@ -2600,7 +2600,7 @@
       </c>
       <c r="F55" s="7" t="inlineStr">
         <is>
-          <t>-1° Uptilt (facing cells only)</t>
+          <t>-1° Uptilt (Increase Coverage – facing cells only)</t>
         </is>
       </c>
       <c r="G55" s="8" t="inlineStr">
@@ -2627,7 +2627,7 @@
       </c>
       <c r="D56" s="10" t="inlineStr">
         <is>
-          <t>+2° Downtilt</t>
+          <t>+2° Downtilt (Reduce Coverage)</t>
         </is>
       </c>
       <c r="E56" s="10" t="inlineStr">
@@ -2664,12 +2664,12 @@
       </c>
       <c r="D57" s="10" t="inlineStr">
         <is>
-          <t>-2° Uptilt</t>
+          <t>-2° Uptilt (Increase Coverage)</t>
         </is>
       </c>
       <c r="E57" s="10" t="inlineStr">
         <is>
-          <t>-1° Uptilt</t>
+          <t>-1° Uptilt (Increase Coverage)</t>
         </is>
       </c>
       <c r="F57" s="10" t="inlineStr">
@@ -2701,7 +2701,7 @@
       </c>
       <c r="D58" s="7" t="inlineStr">
         <is>
-          <t>+1° Downtilt</t>
+          <t>+1° Downtilt (Reduce Coverage)</t>
         </is>
       </c>
       <c r="E58" s="7" t="inlineStr">
@@ -2738,7 +2738,7 @@
       </c>
       <c r="D59" s="7" t="inlineStr">
         <is>
-          <t>-2° Uptilt</t>
+          <t>-2° Uptilt (Increase Coverage)</t>
         </is>
       </c>
       <c r="E59" s="7" t="inlineStr">
@@ -2748,7 +2748,7 @@
       </c>
       <c r="F59" s="7" t="inlineStr">
         <is>
-          <t>-1° Uptilt (facing cells only)</t>
+          <t>-1° Uptilt (Increase Coverage – facing cells only)</t>
         </is>
       </c>
       <c r="G59" s="8" t="inlineStr">
@@ -2775,17 +2775,17 @@
       </c>
       <c r="D60" s="10" t="inlineStr">
         <is>
-          <t>+2° Downtilt</t>
+          <t>+2° Downtilt (Reduce Coverage)</t>
         </is>
       </c>
       <c r="E60" s="10" t="inlineStr">
         <is>
-          <t>+1° Downtilt</t>
+          <t>+1° Downtilt (Reduce Coverage)</t>
         </is>
       </c>
       <c r="F60" s="10" t="inlineStr">
         <is>
-          <t>+1° Downtilt (facing cells)</t>
+          <t>+1° Downtilt (Reduce Coverage – facing cells)</t>
         </is>
       </c>
       <c r="G60" s="11" t="inlineStr">
@@ -2812,7 +2812,7 @@
       </c>
       <c r="D61" s="10" t="inlineStr">
         <is>
-          <t>-1° Uptilt</t>
+          <t>-1° Uptilt (Increase Coverage)</t>
         </is>
       </c>
       <c r="E61" s="10" t="inlineStr">
@@ -2849,17 +2849,17 @@
       </c>
       <c r="D62" s="10" t="inlineStr">
         <is>
-          <t>+4° Downtilt</t>
+          <t>+4° Downtilt (Reduce Coverage)</t>
         </is>
       </c>
       <c r="E62" s="10" t="inlineStr">
         <is>
-          <t>+2° Downtilt</t>
+          <t>+2° Downtilt (Reduce Coverage)</t>
         </is>
       </c>
       <c r="F62" s="10" t="inlineStr">
         <is>
-          <t>+1° Downtilt (facing cells)</t>
+          <t>+1° Downtilt (Reduce Coverage – facing cells)</t>
         </is>
       </c>
       <c r="G62" s="11" t="inlineStr">
@@ -2886,7 +2886,7 @@
       </c>
       <c r="D63" s="10" t="inlineStr">
         <is>
-          <t>+1° Downtilt</t>
+          <t>+1° Downtilt (Reduce Coverage)</t>
         </is>
       </c>
       <c r="E63" s="10" t="inlineStr">
@@ -2923,17 +2923,17 @@
       </c>
       <c r="D64" s="7" t="inlineStr">
         <is>
-          <t>+4° Downtilt</t>
+          <t>+4° Downtilt (Reduce Coverage)</t>
         </is>
       </c>
       <c r="E64" s="7" t="inlineStr">
         <is>
-          <t>+2° Downtilt</t>
+          <t>+2° Downtilt (Reduce Coverage)</t>
         </is>
       </c>
       <c r="F64" s="7" t="inlineStr">
         <is>
-          <t>+1° Downtilt (facing cells)</t>
+          <t>+1° Downtilt (Reduce Coverage – facing cells)</t>
         </is>
       </c>
       <c r="G64" s="8" t="inlineStr">
@@ -2960,7 +2960,7 @@
       </c>
       <c r="D65" s="7" t="inlineStr">
         <is>
-          <t>+1° Downtilt</t>
+          <t>+1° Downtilt (Reduce Coverage)</t>
         </is>
       </c>
       <c r="E65" s="7" t="inlineStr">
@@ -2970,7 +2970,7 @@
       </c>
       <c r="F65" s="7" t="inlineStr">
         <is>
-          <t>-1° Uptilt (cell covering far edge)</t>
+          <t>-1° Uptilt (Increase Coverage – cell covering far edge)</t>
         </is>
       </c>
       <c r="G65" s="8" t="inlineStr">
@@ -2997,17 +2997,17 @@
       </c>
       <c r="D66" s="10" t="inlineStr">
         <is>
-          <t>+3° Downtilt</t>
+          <t>+3° Downtilt (Reduce Coverage)</t>
         </is>
       </c>
       <c r="E66" s="10" t="inlineStr">
         <is>
-          <t>+1° Downtilt</t>
+          <t>+1° Downtilt (Reduce Coverage)</t>
         </is>
       </c>
       <c r="F66" s="10" t="inlineStr">
         <is>
-          <t>+1° Downtilt (facing cells)</t>
+          <t>+1° Downtilt (Reduce Coverage – facing cells)</t>
         </is>
       </c>
       <c r="G66" s="11" t="inlineStr">
@@ -3044,7 +3044,7 @@
       </c>
       <c r="F67" s="10" t="inlineStr">
         <is>
-          <t>-1° Uptilt (cell covering far edge)</t>
+          <t>-1° Uptilt (Increase Coverage – cell covering far edge)</t>
         </is>
       </c>
       <c r="G67" s="11" t="inlineStr">
@@ -3071,12 +3071,12 @@
       </c>
       <c r="D68" s="7" t="inlineStr">
         <is>
-          <t>+3° Downtilt</t>
+          <t>+3° Downtilt (Reduce Coverage)</t>
         </is>
       </c>
       <c r="E68" s="7" t="inlineStr">
         <is>
-          <t>+1° Downtilt</t>
+          <t>+1° Downtilt (Reduce Coverage)</t>
         </is>
       </c>
       <c r="F68" s="7" t="inlineStr">
@@ -3108,7 +3108,7 @@
       </c>
       <c r="D69" s="7" t="inlineStr">
         <is>
-          <t>-1° Uptilt</t>
+          <t>-1° Uptilt (Increase Coverage)</t>
         </is>
       </c>
       <c r="E69" s="7" t="inlineStr">
@@ -3145,12 +3145,12 @@
       </c>
       <c r="D70" s="10" t="inlineStr">
         <is>
-          <t>+2° Downtilt</t>
+          <t>+2° Downtilt (Reduce Coverage)</t>
         </is>
       </c>
       <c r="E70" s="10" t="inlineStr">
         <is>
-          <t>+1° Downtilt</t>
+          <t>+1° Downtilt (Reduce Coverage)</t>
         </is>
       </c>
       <c r="F70" s="10" t="inlineStr">
@@ -3182,7 +3182,7 @@
       </c>
       <c r="D71" s="10" t="inlineStr">
         <is>
-          <t>-1° Uptilt</t>
+          <t>-1° Uptilt (Increase Coverage)</t>
         </is>
       </c>
       <c r="E71" s="10" t="inlineStr">
@@ -3219,17 +3219,17 @@
       </c>
       <c r="D72" s="7" t="inlineStr">
         <is>
-          <t>+4° Downtilt</t>
+          <t>+4° Downtilt (Reduce Coverage)</t>
         </is>
       </c>
       <c r="E72" s="7" t="inlineStr">
         <is>
-          <t>+2° Downtilt</t>
+          <t>+2° Downtilt (Reduce Coverage)</t>
         </is>
       </c>
       <c r="F72" s="7" t="inlineStr">
         <is>
-          <t>+1° Downtilt (facing cells)</t>
+          <t>+1° Downtilt (Reduce Coverage – facing cells)</t>
         </is>
       </c>
       <c r="G72" s="8" t="inlineStr">

</xml_diff>